<commit_message>
feat: adiciona monitoramento incremental de processos DOU e Anvisa
</commit_message>
<xml_diff>
--- a/backend/config/finalidades/dou_diario/palavras_chave.xlsx
+++ b/backend/config/finalidades/dou_diario/palavras_chave.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projetos_Automacao_BA\informativos\backend\config\finalidades\dou_diario\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projetos_Automacao_BA\DOU_Diario_DEV\backend\config\finalidades\dou_diario\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73F47D3A-F4DF-438A-9BB1-6C1510A2891C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E511F1D-4E68-4B28-92BE-2C189A53D4F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{BF9E4AC7-876E-42D2-87EF-D59B4A8F973B}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="684" uniqueCount="602">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="723" uniqueCount="620">
   <si>
     <t>A02 - Acefato</t>
   </si>
@@ -2012,6 +2012,60 @@
   </si>
   <si>
     <t>25351.060824/202627</t>
+  </si>
+  <si>
+    <t>Coral Super Lavável Antimanchas &amp;Antibactérias</t>
+  </si>
+  <si>
+    <t>25351.005476/2025-44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Novo prazo de validade </t>
+  </si>
+  <si>
+    <t>VIGOROX LS-15</t>
+  </si>
+  <si>
+    <t>25351.589433/2021-85</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inclusão de fabricante </t>
+  </si>
+  <si>
+    <t xml:space="preserve">aguardando publicação </t>
+  </si>
+  <si>
+    <t>VIGOROX LS&amp;D</t>
+  </si>
+  <si>
+    <t>25351.589442/2021-76</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VIGOROX 15 F&amp;V </t>
+  </si>
+  <si>
+    <t>25351.589431/2021-00</t>
+  </si>
+  <si>
+    <t>25351.413100/2023-48</t>
+  </si>
+  <si>
+    <t>25351.413040/2023-63</t>
+  </si>
+  <si>
+    <t>25351.413478/2023-41</t>
+  </si>
+  <si>
+    <t>25351.413682/2023-62</t>
+  </si>
+  <si>
+    <t>25351.412719/2023-35</t>
+  </si>
+  <si>
+    <t>25351.373554/2023-79</t>
+  </si>
+  <si>
+    <t>25351.412992/2023-60</t>
   </si>
 </sst>
 </file>
@@ -2080,13 +2134,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor theme="8" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7"/>
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2119,7 +2173,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -2147,12 +2201,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -5580,7 +5631,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38DC278E-2BD7-4A65-8775-F87722AEE101}">
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="40.33203125" customWidth="1"/>
@@ -5645,8 +5696,31 @@
         <v>543</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="B4" s="12"/>
+    <row r="4" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>555</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>602</v>
+      </c>
+      <c r="C4" t="s">
+        <v>603</v>
+      </c>
+      <c r="D4" t="s">
+        <v>553</v>
+      </c>
+      <c r="E4" t="s">
+        <v>548</v>
+      </c>
+      <c r="F4" t="s">
+        <v>558</v>
+      </c>
+      <c r="G4" t="s">
+        <v>604</v>
+      </c>
+      <c r="H4" t="s">
+        <v>543</v>
+      </c>
     </row>
     <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="12" t="s">
@@ -5759,25 +5833,25 @@
       <c r="A11" s="12"/>
     </row>
     <row r="12" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A12" s="13" t="s">
+      <c r="A12" s="12" t="s">
         <v>567</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" t="s">
         <v>568</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="C12" t="s">
         <v>587</v>
       </c>
-      <c r="D12" s="14" t="s">
+      <c r="D12" t="s">
         <v>553</v>
       </c>
-      <c r="E12" s="14" t="s">
+      <c r="E12" t="s">
         <v>548</v>
       </c>
-      <c r="F12" s="14" t="s">
+      <c r="F12" t="s">
         <v>558</v>
       </c>
-      <c r="G12" s="13" t="s">
+      <c r="G12" s="12" t="s">
         <v>569</v>
       </c>
     </row>
@@ -5808,15 +5882,41 @@
         <v>561</v>
       </c>
     </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>574</v>
+      </c>
+      <c r="B15" t="s">
+        <v>605</v>
+      </c>
+      <c r="C15" t="s">
+        <v>606</v>
+      </c>
+      <c r="D15" t="s">
+        <v>553</v>
+      </c>
+      <c r="E15" t="s">
+        <v>548</v>
+      </c>
+      <c r="F15" t="s">
+        <v>558</v>
+      </c>
+      <c r="G15" t="s">
+        <v>607</v>
+      </c>
+      <c r="H15" t="s">
+        <v>608</v>
+      </c>
+    </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>574</v>
       </c>
       <c r="B16" t="s">
-        <v>573</v>
+        <v>609</v>
       </c>
       <c r="C16" t="s">
-        <v>570</v>
+        <v>610</v>
       </c>
       <c r="D16" t="s">
         <v>553</v>
@@ -5828,10 +5928,10 @@
         <v>558</v>
       </c>
       <c r="G16" t="s">
-        <v>561</v>
+        <v>607</v>
       </c>
       <c r="H16" t="s">
-        <v>575</v>
+        <v>608</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
@@ -5839,10 +5939,10 @@
         <v>574</v>
       </c>
       <c r="B17" t="s">
-        <v>572</v>
+        <v>611</v>
       </c>
       <c r="C17" t="s">
-        <v>571</v>
+        <v>612</v>
       </c>
       <c r="D17" t="s">
         <v>553</v>
@@ -5854,133 +5954,139 @@
         <v>558</v>
       </c>
       <c r="G17" t="s">
+        <v>607</v>
+      </c>
+      <c r="H17" t="s">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>574</v>
+      </c>
+      <c r="B19" t="s">
+        <v>573</v>
+      </c>
+      <c r="C19" t="s">
+        <v>570</v>
+      </c>
+      <c r="D19" t="s">
+        <v>553</v>
+      </c>
+      <c r="E19" t="s">
+        <v>548</v>
+      </c>
+      <c r="F19" t="s">
+        <v>558</v>
+      </c>
+      <c r="G19" t="s">
         <v>561</v>
       </c>
-      <c r="H17" t="s">
+      <c r="H19" t="s">
         <v>575</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" s="14" t="s">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
         <v>574</v>
       </c>
-      <c r="B19" s="14" t="s">
+      <c r="B20" t="s">
+        <v>572</v>
+      </c>
+      <c r="C20" t="s">
+        <v>571</v>
+      </c>
+      <c r="D20" t="s">
+        <v>553</v>
+      </c>
+      <c r="E20" t="s">
+        <v>548</v>
+      </c>
+      <c r="F20" t="s">
+        <v>558</v>
+      </c>
+      <c r="G20" t="s">
+        <v>561</v>
+      </c>
+      <c r="H20" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>574</v>
+      </c>
+      <c r="B22" t="s">
         <v>588</v>
       </c>
-      <c r="C19" s="14" t="s">
+      <c r="C22" t="s">
         <v>589</v>
       </c>
-      <c r="D19" s="14" t="s">
+      <c r="D22" t="s">
         <v>553</v>
       </c>
-      <c r="E19" s="14" t="s">
+      <c r="E22" t="s">
         <v>548</v>
       </c>
-      <c r="F19" s="14" t="s">
+      <c r="F22" t="s">
         <v>558</v>
-      </c>
-      <c r="G19" s="14" t="s">
-        <v>561</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="B21" t="s">
-        <v>578</v>
-      </c>
-      <c r="C21" t="s">
-        <v>579</v>
-      </c>
-      <c r="D21" t="s">
-        <v>553</v>
-      </c>
-      <c r="E21" t="s">
-        <v>548</v>
-      </c>
-      <c r="F21" t="s">
-        <v>580</v>
-      </c>
-      <c r="G21" t="s">
-        <v>561</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B22" t="s">
-        <v>578</v>
-      </c>
-      <c r="C22" t="s">
-        <v>581</v>
-      </c>
-      <c r="D22" s="12" t="s">
-        <v>554</v>
-      </c>
-      <c r="E22" t="s">
-        <v>550</v>
-      </c>
-      <c r="F22" t="s">
-        <v>559</v>
       </c>
       <c r="G22" t="s">
         <v>561</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="B23" t="s">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B24" t="s">
         <v>578</v>
       </c>
-      <c r="C23" t="s">
-        <v>582</v>
-      </c>
-      <c r="D23" t="s">
-        <v>551</v>
-      </c>
-      <c r="E23" t="s">
-        <v>547</v>
-      </c>
-      <c r="F23" t="s">
+      <c r="C24" t="s">
+        <v>579</v>
+      </c>
+      <c r="D24" t="s">
+        <v>553</v>
+      </c>
+      <c r="E24" t="s">
+        <v>548</v>
+      </c>
+      <c r="F24" t="s">
+        <v>580</v>
+      </c>
+      <c r="G24" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B25" t="s">
+        <v>578</v>
+      </c>
+      <c r="C25" t="s">
+        <v>581</v>
+      </c>
+      <c r="D25" s="12" t="s">
+        <v>554</v>
+      </c>
+      <c r="E25" t="s">
+        <v>550</v>
+      </c>
+      <c r="F25" t="s">
         <v>559</v>
-      </c>
-      <c r="G23" t="s">
-        <v>561</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>590</v>
-      </c>
-      <c r="B25" t="s">
-        <v>583</v>
-      </c>
-      <c r="C25" t="s">
-        <v>584</v>
-      </c>
-      <c r="D25" t="s">
-        <v>553</v>
-      </c>
-      <c r="E25" t="s">
-        <v>548</v>
-      </c>
-      <c r="F25" t="s">
-        <v>580</v>
       </c>
       <c r="G25" t="s">
         <v>561</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>590</v>
-      </c>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
-        <v>583</v>
+        <v>578</v>
       </c>
       <c r="C26" t="s">
-        <v>585</v>
-      </c>
-      <c r="D26" s="12" t="s">
-        <v>554</v>
+        <v>582</v>
+      </c>
+      <c r="D26" t="s">
+        <v>551</v>
       </c>
       <c r="E26" t="s">
-        <v>550</v>
+        <v>547</v>
       </c>
       <c r="F26" t="s">
         <v>559</v>
@@ -5989,108 +6095,186 @@
         <v>561</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
         <v>590</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B28" t="s">
         <v>583</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C28" t="s">
+        <v>584</v>
+      </c>
+      <c r="D28" t="s">
+        <v>553</v>
+      </c>
+      <c r="E28" t="s">
+        <v>548</v>
+      </c>
+      <c r="F28" t="s">
+        <v>580</v>
+      </c>
+      <c r="G28" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>590</v>
+      </c>
+      <c r="B29" t="s">
+        <v>583</v>
+      </c>
+      <c r="C29" t="s">
+        <v>585</v>
+      </c>
+      <c r="D29" s="12" t="s">
+        <v>554</v>
+      </c>
+      <c r="E29" t="s">
+        <v>550</v>
+      </c>
+      <c r="F29" t="s">
+        <v>559</v>
+      </c>
+      <c r="G29" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>590</v>
+      </c>
+      <c r="B30" t="s">
+        <v>583</v>
+      </c>
+      <c r="C30" t="s">
         <v>586</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D30" t="s">
         <v>551</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E30" t="s">
         <v>547</v>
       </c>
-      <c r="F27" t="s">
+      <c r="F30" t="s">
         <v>559</v>
       </c>
-      <c r="G27" t="s">
+      <c r="G30" t="s">
         <v>561</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A29" s="14" t="s">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
         <v>591</v>
       </c>
-      <c r="B29" s="14" t="s">
+      <c r="B32" t="s">
         <v>592</v>
       </c>
-      <c r="C29" s="15" t="s">
+      <c r="C32" s="13" t="s">
         <v>593</v>
       </c>
-      <c r="D29" s="14" t="s">
+      <c r="D32" t="s">
         <v>553</v>
       </c>
-      <c r="E29" s="14" t="s">
+      <c r="E32" t="s">
         <v>548</v>
       </c>
-      <c r="F29" s="14" t="s">
+      <c r="F32" t="s">
         <v>594</v>
       </c>
-      <c r="G29" s="14" t="s">
+      <c r="G32" t="s">
         <v>595</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A30" s="14" t="s">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
         <v>591</v>
       </c>
-      <c r="B30" s="14" t="s">
+      <c r="B33" t="s">
         <v>596</v>
       </c>
-      <c r="C30" s="14" t="s">
+      <c r="C33" t="s">
         <v>597</v>
       </c>
-      <c r="D30" s="14" t="s">
+      <c r="D33" t="s">
         <v>553</v>
       </c>
-      <c r="E30" s="14" t="s">
+      <c r="E33" t="s">
         <v>548</v>
       </c>
-      <c r="F30" s="14" t="s">
+      <c r="F33" t="s">
         <v>594</v>
       </c>
-      <c r="G30" s="14" t="s">
+      <c r="G33" t="s">
         <v>595</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A32" s="14" t="s">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
         <v>598</v>
       </c>
-      <c r="B32" s="16" t="s">
+      <c r="B35" s="14" t="s">
         <v>599</v>
       </c>
-      <c r="C32" s="14" t="s">
+      <c r="C35" t="s">
         <v>600</v>
       </c>
-      <c r="D32" s="14" t="s">
+      <c r="D35" t="s">
         <v>553</v>
       </c>
-      <c r="E32" s="14" t="s">
+      <c r="E35" t="s">
         <v>548</v>
       </c>
-      <c r="F32" s="14" t="s">
+      <c r="F35" t="s">
         <v>558</v>
       </c>
-      <c r="G32" s="14" t="s">
+      <c r="G35" t="s">
         <v>561</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A34" s="17"/>
-      <c r="B34" s="17"/>
-      <c r="C34" s="17" t="s">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C37" t="s">
         <v>601</v>
       </c>
-      <c r="D34" s="17"/>
-      <c r="E34" s="17"/>
-      <c r="F34" s="17"/>
-      <c r="G34" s="17"/>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C39" s="15" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C40" s="15" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C41" s="15" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C42" s="15" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C43" s="15" t="s">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C44" s="15" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C45" s="15" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C47" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
Atualiza planilha de palavras-chave com novos processos
</commit_message>
<xml_diff>
--- a/backend/config/finalidades/dou_diario/palavras_chave.xlsx
+++ b/backend/config/finalidades/dou_diario/palavras_chave.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projetos_Automacao_BA\DOU_Diario_DEV\backend\config\finalidades\dou_diario\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projetos_Automacao_BA\DOU_Diario_PROD\backend\config\finalidades\dou_diario\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E511F1D-4E68-4B28-92BE-2C189A53D4F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4F85CD6-9AF5-482E-8E69-4D46841E58D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{BF9E4AC7-876E-42D2-87EF-D59B4A8F973B}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="723" uniqueCount="620">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="738" uniqueCount="626">
   <si>
     <t>A02 - Acefato</t>
   </si>
@@ -2066,6 +2066,24 @@
   </si>
   <si>
     <t>25351.412992/2023-60</t>
+  </si>
+  <si>
+    <t>PYRIMETHANIL</t>
+  </si>
+  <si>
+    <t>21000.071679/2026-39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRANSFERÊNCIA DE TITULARIDADE </t>
+  </si>
+  <si>
+    <t>SHARDA DO BRASIL</t>
+  </si>
+  <si>
+    <t>QUIZALOFOP</t>
+  </si>
+  <si>
+    <t>21000.071680/2026-63</t>
   </si>
 </sst>
 </file>
@@ -2173,7 +2191,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -2205,6 +2223,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
@@ -5631,7 +5652,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38DC278E-2BD7-4A65-8775-F87722AEE101}">
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="40.33203125" customWidth="1"/>
@@ -6187,7 +6208,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>591</v>
       </c>
@@ -6210,7 +6231,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>598</v>
       </c>
@@ -6233,48 +6254,94 @@
         <v>561</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C37" t="s">
         <v>601</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C39" s="15" t="s">
         <v>613</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C40" s="15" t="s">
         <v>614</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C41" s="15" t="s">
         <v>615</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C42" s="15" t="s">
         <v>616</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C43" s="15" t="s">
         <v>617</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C44" s="15" t="s">
         <v>618</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C45" s="15" t="s">
         <v>619</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C47" s="16"/>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>623</v>
+      </c>
+      <c r="B47" s="17" t="s">
+        <v>620</v>
+      </c>
+      <c r="C47" s="16" t="s">
+        <v>621</v>
+      </c>
+      <c r="D47" s="16" t="s">
+        <v>551</v>
+      </c>
+      <c r="E47" s="16" t="s">
+        <v>547</v>
+      </c>
+      <c r="F47" s="16" t="s">
+        <v>559</v>
+      </c>
+      <c r="G47" s="16" t="s">
+        <v>622</v>
+      </c>
+      <c r="H47" s="16" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="49" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B49" s="17" t="s">
+        <v>624</v>
+      </c>
+      <c r="C49" s="16" t="s">
+        <v>625</v>
+      </c>
+      <c r="D49" s="16" t="s">
+        <v>551</v>
+      </c>
+      <c r="E49" s="16" t="s">
+        <v>547</v>
+      </c>
+      <c r="F49" s="16" t="s">
+        <v>559</v>
+      </c>
+      <c r="G49" s="16" t="s">
+        <v>622</v>
+      </c>
+      <c r="H49" s="16" t="s">
+        <v>543</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>